<commit_message>
fix ProductionSource.name & technology requirements
</commit_message>
<xml_diff>
--- a/docs/PEACH_DataModel.xlsx
+++ b/docs/PEACH_DataModel.xlsx
@@ -54,7 +54,21 @@
     <t>Version Date</t>
   </si>
   <si>
-    <t>2026-01-14</t>
+    <r>
+      <rPr/>
+      <t xml:space="preserve">2026-01-19    (for updates refer to the </t>
+    </r>
+    <r>
+      <rPr>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>changelog</t>
+    </r>
+    <r>
+      <rPr/>
+      <t>)</t>
+    </r>
   </si>
   <si>
     <t>Key Architecture Principle</t>
@@ -1930,7 +1944,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <sz val="11.0"/>
       <color theme="1"/>
@@ -1955,6 +1969,10 @@
       <color theme="1"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <color rgb="FF0000FF"/>
     </font>
     <font>
       <b/>
@@ -2029,24 +2047,30 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="1" fillId="2" fontId="2" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="1" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0"/>
+    </xf>
+    <xf borderId="1" fillId="3" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="top" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="2" fillId="2" fontId="7" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="3" fillId="0" fontId="8" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="4" fillId="0" fontId="8" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="1" fillId="3" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="top" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="2" fillId="2" fontId="8" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="3" fillId="0" fontId="9" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="4" fillId="0" fontId="9" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="1" fillId="3" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -2347,7 +2371,7 @@
       <c r="A7" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="4" t="s">
         <v>8</v>
       </c>
     </row>
@@ -3464,10 +3488,13 @@
     <row r="999" ht="15.75" customHeight="1"/>
     <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
+  <hyperlinks>
+    <hyperlink r:id="rId1" ref="B7"/>
+  </hyperlinks>
   <printOptions/>
   <pageMargins bottom="1.0" footer="0.0" header="0.0" left="0.75" right="0.75" top="1.0"/>
   <pageSetup orientation="landscape"/>
-  <drawing r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -3489,239 +3516,239 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="G1" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="H1" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="I1" s="5" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="6" t="s">
         <v>413</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="C2" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="D2" s="6" t="s">
         <v>414</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="E2" s="6" t="s">
         <v>415</v>
       </c>
-      <c r="F2" s="5"/>
-      <c r="G2" s="5" t="s">
+      <c r="F2" s="6"/>
+      <c r="G2" s="6" t="s">
         <v>416</v>
       </c>
-      <c r="H2" s="5" t="s">
+      <c r="H2" s="6" t="s">
         <v>417</v>
       </c>
-      <c r="I2" s="5" t="s">
+      <c r="I2" s="6" t="s">
         <v>418</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="6" t="s">
         <v>419</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="6" t="s">
         <v>420</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="E3" s="6" t="s">
         <v>421</v>
       </c>
-      <c r="F3" s="5"/>
-      <c r="G3" s="5" t="s">
+      <c r="F3" s="6"/>
+      <c r="G3" s="6" t="s">
         <v>422</v>
       </c>
-      <c r="H3" s="5" t="s">
+      <c r="H3" s="6" t="s">
         <v>423</v>
       </c>
-      <c r="I3" s="5"/>
+      <c r="I3" s="6"/>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="6" t="s">
         <v>424</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="6" t="s">
         <v>425</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="E4" s="6" t="s">
         <v>426</v>
       </c>
-      <c r="F4" s="5"/>
-      <c r="G4" s="5" t="s">
+      <c r="F4" s="6"/>
+      <c r="G4" s="6" t="s">
         <v>427</v>
       </c>
-      <c r="H4" s="5" t="s">
+      <c r="H4" s="6" t="s">
         <v>428</v>
       </c>
-      <c r="I4" s="5"/>
+      <c r="I4" s="6"/>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="6" t="s">
         <v>429</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D5" s="6" t="s">
         <v>430</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="E5" s="6" t="s">
         <v>431</v>
       </c>
-      <c r="F5" s="5"/>
-      <c r="G5" s="5" t="s">
+      <c r="F5" s="6"/>
+      <c r="G5" s="6" t="s">
         <v>432</v>
       </c>
-      <c r="H5" s="5" t="s">
+      <c r="H5" s="6" t="s">
         <v>433</v>
       </c>
-      <c r="I5" s="5" t="s">
+      <c r="I5" s="6" t="s">
         <v>434</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="6" t="s">
         <v>435</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="D6" s="6" t="s">
         <v>436</v>
       </c>
-      <c r="E6" s="5" t="s">
+      <c r="E6" s="6" t="s">
         <v>185</v>
       </c>
-      <c r="F6" s="5"/>
-      <c r="G6" s="5" t="s">
+      <c r="F6" s="6"/>
+      <c r="G6" s="6" t="s">
         <v>437</v>
       </c>
-      <c r="H6" s="5" t="s">
+      <c r="H6" s="6" t="s">
         <v>438</v>
       </c>
-      <c r="I6" s="5" t="s">
+      <c r="I6" s="6" t="s">
         <v>439</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="s">
+      <c r="A7" s="6" t="s">
         <v>440</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="6" t="s">
         <v>355</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="C7" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="D7" s="6" t="s">
         <v>441</v>
       </c>
-      <c r="E7" s="5" t="s">
+      <c r="E7" s="6" t="s">
         <v>442</v>
       </c>
-      <c r="F7" s="5"/>
-      <c r="G7" s="5" t="s">
+      <c r="F7" s="6"/>
+      <c r="G7" s="6" t="s">
         <v>443</v>
       </c>
-      <c r="H7" s="5" t="s">
+      <c r="H7" s="6" t="s">
         <v>444</v>
       </c>
-      <c r="I7" s="5" t="s">
+      <c r="I7" s="6" t="s">
         <v>445</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="s">
+      <c r="A8" s="6" t="s">
         <v>446</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="6" t="s">
         <v>355</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="C8" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="D8" s="6" t="s">
         <v>447</v>
       </c>
-      <c r="E8" s="5" t="s">
+      <c r="E8" s="6" t="s">
         <v>448</v>
       </c>
-      <c r="F8" s="5"/>
-      <c r="G8" s="5" t="s">
+      <c r="F8" s="6"/>
+      <c r="G8" s="6" t="s">
         <v>449</v>
       </c>
-      <c r="H8" s="5" t="s">
+      <c r="H8" s="6" t="s">
         <v>450</v>
       </c>
-      <c r="I8" s="5" t="s">
+      <c r="I8" s="6" t="s">
         <v>451</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="s">
+      <c r="A9" s="6" t="s">
         <v>452</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="C9" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="D9" s="5" t="s">
+      <c r="D9" s="6" t="s">
         <v>453</v>
       </c>
-      <c r="E9" s="5" t="s">
+      <c r="E9" s="6" t="s">
         <v>454</v>
       </c>
-      <c r="F9" s="5"/>
-      <c r="G9" s="5"/>
-      <c r="H9" s="5"/>
-      <c r="I9" s="5"/>
+      <c r="F9" s="6"/>
+      <c r="G9" s="6"/>
+      <c r="H9" s="6"/>
+      <c r="I9" s="6"/>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
     <row r="22" ht="15.75" customHeight="1"/>
@@ -4730,204 +4757,204 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="G1" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="H1" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="I1" s="5" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="6" t="s">
         <v>455</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="C2" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="D2" s="6" t="s">
         <v>456</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="E2" s="6" t="s">
         <v>457</v>
       </c>
-      <c r="F2" s="5"/>
-      <c r="G2" s="5"/>
-      <c r="H2" s="5" t="s">
+      <c r="F2" s="6"/>
+      <c r="G2" s="6"/>
+      <c r="H2" s="6" t="s">
         <v>458</v>
       </c>
-      <c r="I2" s="5" t="s">
+      <c r="I2" s="6" t="s">
         <v>459</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="6" t="s">
         <v>460</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="6" t="s">
         <v>461</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="E3" s="6" t="s">
         <v>185</v>
       </c>
-      <c r="F3" s="5"/>
-      <c r="G3" s="5"/>
-      <c r="H3" s="5" t="s">
+      <c r="F3" s="6"/>
+      <c r="G3" s="6"/>
+      <c r="H3" s="6" t="s">
         <v>462</v>
       </c>
-      <c r="I3" s="5" t="s">
+      <c r="I3" s="6" t="s">
         <v>463</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="6" t="s">
         <v>189</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="6" t="s">
         <v>464</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="E4" s="6" t="s">
         <v>465</v>
       </c>
-      <c r="F4" s="5"/>
-      <c r="G4" s="5"/>
-      <c r="H4" s="5" t="s">
+      <c r="F4" s="6"/>
+      <c r="G4" s="6"/>
+      <c r="H4" s="6" t="s">
         <v>466</v>
       </c>
-      <c r="I4" s="5" t="s">
+      <c r="I4" s="6" t="s">
         <v>467</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D5" s="6" t="s">
         <v>468</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="E5" s="6" t="s">
         <v>469</v>
       </c>
-      <c r="F5" s="5"/>
-      <c r="G5" s="5"/>
-      <c r="H5" s="5" t="s">
+      <c r="F5" s="6"/>
+      <c r="G5" s="6"/>
+      <c r="H5" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="I5" s="5" t="s">
+      <c r="I5" s="6" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="6" t="s">
         <v>470</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="6" t="s">
         <v>126</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="D6" s="6" t="s">
         <v>471</v>
       </c>
-      <c r="E6" s="5" t="s">
+      <c r="E6" s="6" t="s">
         <v>472</v>
       </c>
-      <c r="F6" s="5"/>
-      <c r="G6" s="5"/>
-      <c r="H6" s="5"/>
-      <c r="I6" s="5" t="s">
+      <c r="F6" s="6"/>
+      <c r="G6" s="6"/>
+      <c r="H6" s="6"/>
+      <c r="I6" s="6" t="s">
         <v>473</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="s">
+      <c r="A7" s="6" t="s">
         <v>474</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="6" t="s">
         <v>381</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="C7" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="D7" s="6" t="s">
         <v>475</v>
       </c>
-      <c r="E7" s="5" t="s">
+      <c r="E7" s="6" t="s">
         <v>383</v>
       </c>
-      <c r="F7" s="5"/>
-      <c r="G7" s="5"/>
-      <c r="H7" s="5" t="s">
+      <c r="F7" s="6"/>
+      <c r="G7" s="6"/>
+      <c r="H7" s="6" t="s">
         <v>476</v>
       </c>
-      <c r="I7" s="5" t="s">
+      <c r="I7" s="6" t="s">
         <v>384</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="s">
+      <c r="A8" s="6" t="s">
         <v>229</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="C8" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="D8" s="6" t="s">
         <v>477</v>
       </c>
-      <c r="E8" s="5" t="s">
+      <c r="E8" s="6" t="s">
         <v>185</v>
       </c>
-      <c r="F8" s="5"/>
-      <c r="G8" s="5"/>
-      <c r="H8" s="5" t="s">
+      <c r="F8" s="6"/>
+      <c r="G8" s="6"/>
+      <c r="H8" s="6" t="s">
         <v>478</v>
       </c>
-      <c r="I8" s="5" t="s">
+      <c r="I8" s="6" t="s">
         <v>479</v>
       </c>
     </row>
@@ -5938,168 +5965,168 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="G1" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="H1" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="I1" s="5" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="C2" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="D2" s="6" t="s">
         <v>480</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="E2" s="6" t="s">
         <v>185</v>
       </c>
-      <c r="F2" s="5"/>
-      <c r="G2" s="5" t="s">
+      <c r="F2" s="6"/>
+      <c r="G2" s="6" t="s">
         <v>481</v>
       </c>
-      <c r="H2" s="5" t="s">
+      <c r="H2" s="6" t="s">
         <v>482</v>
       </c>
-      <c r="I2" s="5" t="s">
+      <c r="I2" s="6" t="s">
         <v>483</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="6" t="s">
         <v>484</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="6" t="s">
         <v>485</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="E3" s="6" t="s">
         <v>337</v>
       </c>
-      <c r="F3" s="5" t="s">
+      <c r="F3" s="6" t="s">
         <v>196</v>
       </c>
-      <c r="G3" s="5" t="s">
+      <c r="G3" s="6" t="s">
         <v>303</v>
       </c>
-      <c r="H3" s="5" t="s">
+      <c r="H3" s="6" t="s">
         <v>304</v>
       </c>
-      <c r="I3" s="5" t="s">
+      <c r="I3" s="6" t="s">
         <v>305</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="6" t="s">
         <v>486</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="6" t="s">
         <v>487</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="E4" s="6" t="s">
         <v>185</v>
       </c>
-      <c r="F4" s="5"/>
-      <c r="G4" s="5" t="s">
+      <c r="F4" s="6"/>
+      <c r="G4" s="6" t="s">
         <v>307</v>
       </c>
-      <c r="H4" s="5" t="s">
+      <c r="H4" s="6" t="s">
         <v>308</v>
       </c>
-      <c r="I4" s="5" t="s">
+      <c r="I4" s="6" t="s">
         <v>488</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="6" t="s">
         <v>229</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D5" s="6" t="s">
         <v>489</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="E5" s="6" t="s">
         <v>185</v>
       </c>
-      <c r="F5" s="5"/>
-      <c r="G5" s="5" t="s">
+      <c r="F5" s="6"/>
+      <c r="G5" s="6" t="s">
         <v>490</v>
       </c>
-      <c r="H5" s="5" t="s">
+      <c r="H5" s="6" t="s">
         <v>491</v>
       </c>
-      <c r="I5" s="5" t="s">
+      <c r="I5" s="6" t="s">
         <v>492</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="6" t="s">
         <v>493</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="D6" s="6" t="s">
         <v>494</v>
       </c>
-      <c r="E6" s="5" t="s">
+      <c r="E6" s="6" t="s">
         <v>185</v>
       </c>
-      <c r="F6" s="5"/>
-      <c r="G6" s="5" t="s">
+      <c r="F6" s="6"/>
+      <c r="G6" s="6" t="s">
         <v>495</v>
       </c>
-      <c r="H6" s="5" t="s">
+      <c r="H6" s="6" t="s">
         <v>496</v>
       </c>
-      <c r="I6" s="5" t="s">
+      <c r="I6" s="6" t="s">
         <v>497</v>
       </c>
     </row>
@@ -7105,25 +7132,25 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="8" t="s">
         <v>498</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="s">
+      <c r="A3" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="B3" s="8"/>
-      <c r="C3" s="9"/>
+      <c r="B3" s="10"/>
+      <c r="C3" s="11"/>
     </row>
     <row r="4">
-      <c r="A4" s="10" t="s">
+      <c r="A4" s="12" t="s">
         <v>499</v>
       </c>
-      <c r="B4" s="10" t="s">
+      <c r="B4" s="12" t="s">
         <v>500</v>
       </c>
-      <c r="C4" s="10" t="s">
+      <c r="C4" s="12" t="s">
         <v>44</v>
       </c>
     </row>
@@ -7183,20 +7210,20 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="s">
+      <c r="A12" s="9" t="s">
         <v>150</v>
       </c>
-      <c r="B12" s="8"/>
-      <c r="C12" s="9"/>
+      <c r="B12" s="10"/>
+      <c r="C12" s="11"/>
     </row>
     <row r="13">
-      <c r="A13" s="10" t="s">
+      <c r="A13" s="12" t="s">
         <v>499</v>
       </c>
-      <c r="B13" s="10" t="s">
+      <c r="B13" s="12" t="s">
         <v>500</v>
       </c>
-      <c r="C13" s="10" t="s">
+      <c r="C13" s="12" t="s">
         <v>44</v>
       </c>
     </row>
@@ -7401,20 +7428,20 @@
     <row r="32" ht="15.75" customHeight="1"/>
     <row r="33" ht="15.75" customHeight="1"/>
     <row r="34" ht="15.75" customHeight="1">
-      <c r="A34" s="7" t="s">
+      <c r="A34" s="9" t="s">
         <v>157</v>
       </c>
-      <c r="B34" s="8"/>
-      <c r="C34" s="9"/>
+      <c r="B34" s="10"/>
+      <c r="C34" s="11"/>
     </row>
     <row r="35" ht="15.75" customHeight="1">
-      <c r="A35" s="10" t="s">
+      <c r="A35" s="12" t="s">
         <v>499</v>
       </c>
-      <c r="B35" s="10" t="s">
+      <c r="B35" s="12" t="s">
         <v>500</v>
       </c>
-      <c r="C35" s="10" t="s">
+      <c r="C35" s="12" t="s">
         <v>44</v>
       </c>
     </row>
@@ -7454,20 +7481,20 @@
     <row r="39" ht="15.75" customHeight="1"/>
     <row r="40" ht="15.75" customHeight="1"/>
     <row r="41" ht="15.75" customHeight="1">
-      <c r="A41" s="7" t="s">
+      <c r="A41" s="9" t="s">
         <v>345</v>
       </c>
-      <c r="B41" s="8"/>
-      <c r="C41" s="9"/>
+      <c r="B41" s="10"/>
+      <c r="C41" s="11"/>
     </row>
     <row r="42" ht="15.75" customHeight="1">
-      <c r="A42" s="10" t="s">
+      <c r="A42" s="12" t="s">
         <v>499</v>
       </c>
-      <c r="B42" s="10" t="s">
+      <c r="B42" s="12" t="s">
         <v>500</v>
       </c>
-      <c r="C42" s="10" t="s">
+      <c r="C42" s="12" t="s">
         <v>44</v>
       </c>
     </row>
@@ -7661,20 +7688,20 @@
     <row r="60" ht="15.75" customHeight="1"/>
     <row r="61" ht="15.75" customHeight="1"/>
     <row r="62" ht="15.75" customHeight="1">
-      <c r="A62" s="7" t="s">
+      <c r="A62" s="9" t="s">
         <v>285</v>
       </c>
-      <c r="B62" s="8"/>
-      <c r="C62" s="9"/>
+      <c r="B62" s="10"/>
+      <c r="C62" s="11"/>
     </row>
     <row r="63" ht="15.75" customHeight="1">
-      <c r="A63" s="10" t="s">
+      <c r="A63" s="12" t="s">
         <v>499</v>
       </c>
-      <c r="B63" s="10" t="s">
+      <c r="B63" s="12" t="s">
         <v>500</v>
       </c>
-      <c r="C63" s="10" t="s">
+      <c r="C63" s="12" t="s">
         <v>44</v>
       </c>
     </row>
@@ -8718,398 +8745,398 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="G1" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="H1" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="I1" s="5" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="C2" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="D2" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="E2" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="F2" s="5"/>
-      <c r="G2" s="5" t="s">
+      <c r="F2" s="6"/>
+      <c r="G2" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="H2" s="5" t="s">
+      <c r="H2" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="I2" s="5" t="s">
+      <c r="I2" s="6" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="E3" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="F3" s="5" t="s">
+      <c r="F3" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="G3" s="5" t="s">
+      <c r="G3" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="H3" s="5" t="s">
+      <c r="H3" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="I3" s="5" t="s">
+      <c r="I3" s="6" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="E4" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="F4" s="5"/>
-      <c r="G4" s="5" t="s">
+      <c r="F4" s="6"/>
+      <c r="G4" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="H4" s="5" t="s">
+      <c r="H4" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="I4" s="5" t="s">
+      <c r="I4" s="6" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D5" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="E5" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="F5" s="5" t="s">
+      <c r="F5" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="G5" s="5" t="s">
+      <c r="G5" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="H5" s="5" t="s">
+      <c r="H5" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="I5" s="5" t="s">
+      <c r="I5" s="6" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="D6" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="E6" s="5" t="s">
+      <c r="E6" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="F6" s="5" t="s">
+      <c r="F6" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="G6" s="5" t="s">
+      <c r="G6" s="6" t="s">
         <v>84</v>
       </c>
-      <c r="H6" s="5" t="s">
+      <c r="H6" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="I6" s="5" t="s">
+      <c r="I6" s="6" t="s">
         <v>86</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="s">
+      <c r="A7" s="6" t="s">
         <v>87</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="C7" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="D7" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="E7" s="5" t="s">
+      <c r="E7" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="F7" s="5" t="s">
+      <c r="F7" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="G7" s="5" t="s">
+      <c r="G7" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="H7" s="5" t="s">
+      <c r="H7" s="6" t="s">
         <v>93</v>
       </c>
-      <c r="I7" s="5" t="s">
+      <c r="I7" s="6" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="s">
+      <c r="A8" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="C8" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="D8" s="6" t="s">
         <v>97</v>
       </c>
-      <c r="E8" s="5" t="s">
+      <c r="E8" s="6" t="s">
         <v>98</v>
       </c>
-      <c r="F8" s="5" t="s">
+      <c r="F8" s="6" t="s">
         <v>99</v>
       </c>
-      <c r="G8" s="5" t="s">
+      <c r="G8" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="H8" s="5" t="s">
+      <c r="H8" s="6" t="s">
         <v>101</v>
       </c>
-      <c r="I8" s="5" t="s">
+      <c r="I8" s="6" t="s">
         <v>102</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="s">
+      <c r="A9" s="6" t="s">
         <v>103</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="C9" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="D9" s="5" t="s">
+      <c r="D9" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="E9" s="5" t="s">
+      <c r="E9" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="F9" s="5"/>
-      <c r="G9" s="5" t="s">
+      <c r="F9" s="6"/>
+      <c r="G9" s="6" t="s">
         <v>106</v>
       </c>
-      <c r="H9" s="5" t="s">
+      <c r="H9" s="6" t="s">
         <v>107</v>
       </c>
-      <c r="I9" s="5" t="s">
+      <c r="I9" s="6" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="s">
+      <c r="A10" s="6" t="s">
         <v>109</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="B10" s="6" t="s">
         <v>110</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="C10" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="D10" s="5" t="s">
+      <c r="D10" s="6" t="s">
         <v>111</v>
       </c>
-      <c r="E10" s="5" t="s">
+      <c r="E10" s="6" t="s">
         <v>112</v>
       </c>
-      <c r="F10" s="5" t="s">
+      <c r="F10" s="6" t="s">
         <v>113</v>
       </c>
-      <c r="G10" s="5" t="s">
+      <c r="G10" s="6" t="s">
         <v>114</v>
       </c>
-      <c r="H10" s="5" t="s">
+      <c r="H10" s="6" t="s">
         <v>115</v>
       </c>
-      <c r="I10" s="5" t="s">
+      <c r="I10" s="6" t="s">
         <v>116</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="s">
+      <c r="A11" s="6" t="s">
         <v>117</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="B11" s="6" t="s">
         <v>118</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="C11" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="D11" s="5" t="s">
+      <c r="D11" s="6" t="s">
         <v>119</v>
       </c>
-      <c r="E11" s="5" t="s">
+      <c r="E11" s="6" t="s">
         <v>120</v>
       </c>
-      <c r="F11" s="5" t="s">
+      <c r="F11" s="6" t="s">
         <v>121</v>
       </c>
-      <c r="G11" s="5" t="s">
+      <c r="G11" s="6" t="s">
         <v>122</v>
       </c>
-      <c r="H11" s="5" t="s">
+      <c r="H11" s="6" t="s">
         <v>123</v>
       </c>
-      <c r="I11" s="5" t="s">
+      <c r="I11" s="6" t="s">
         <v>124</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="s">
+      <c r="A12" s="6" t="s">
         <v>125</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="B12" s="6" t="s">
         <v>126</v>
       </c>
-      <c r="C12" s="5" t="s">
+      <c r="C12" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="D12" s="5" t="s">
+      <c r="D12" s="6" t="s">
         <v>127</v>
       </c>
-      <c r="E12" s="5" t="s">
+      <c r="E12" s="6" t="s">
         <v>128</v>
       </c>
-      <c r="F12" s="5"/>
-      <c r="G12" s="5" t="s">
+      <c r="F12" s="6"/>
+      <c r="G12" s="6" t="s">
         <v>129</v>
       </c>
-      <c r="H12" s="5" t="s">
+      <c r="H12" s="6" t="s">
         <v>130</v>
       </c>
-      <c r="I12" s="5" t="s">
+      <c r="I12" s="6" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="s">
+      <c r="A13" s="6" t="s">
         <v>131</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="B13" s="6" t="s">
         <v>126</v>
       </c>
-      <c r="C13" s="5" t="s">
+      <c r="C13" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="D13" s="5" t="s">
+      <c r="D13" s="6" t="s">
         <v>132</v>
       </c>
-      <c r="E13" s="5" t="s">
+      <c r="E13" s="6" t="s">
         <v>133</v>
       </c>
-      <c r="F13" s="5"/>
-      <c r="G13" s="5" t="s">
+      <c r="F13" s="6"/>
+      <c r="G13" s="6" t="s">
         <v>134</v>
       </c>
-      <c r="H13" s="5" t="s">
+      <c r="H13" s="6" t="s">
         <v>135</v>
       </c>
-      <c r="I13" s="5" t="s">
+      <c r="I13" s="6" t="s">
         <v>136</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="s">
+      <c r="A14" s="6" t="s">
         <v>137</v>
       </c>
-      <c r="B14" s="5" t="s">
+      <c r="B14" s="6" t="s">
         <v>138</v>
       </c>
-      <c r="C14" s="5" t="s">
+      <c r="C14" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="D14" s="5" t="s">
+      <c r="D14" s="6" t="s">
         <v>139</v>
       </c>
-      <c r="E14" s="5" t="s">
+      <c r="E14" s="6" t="s">
         <v>140</v>
       </c>
-      <c r="F14" s="5" t="s">
+      <c r="F14" s="6" t="s">
         <v>141</v>
       </c>
-      <c r="G14" s="5" t="s">
+      <c r="G14" s="6" t="s">
         <v>142</v>
       </c>
-      <c r="H14" s="5" t="s">
+      <c r="H14" s="6" t="s">
         <v>143</v>
       </c>
-      <c r="I14" s="5" t="s">
+      <c r="I14" s="6" t="s">
         <v>142</v>
       </c>
     </row>
@@ -10118,334 +10145,334 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="G1" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="H1" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="I1" s="5" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="C2" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="D2" s="6" t="s">
         <v>144</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="E2" s="6" t="s">
         <v>145</v>
       </c>
-      <c r="F2" s="5"/>
-      <c r="G2" s="5" t="s">
+      <c r="F2" s="6"/>
+      <c r="G2" s="6" t="s">
         <v>146</v>
       </c>
-      <c r="H2" s="5" t="s">
+      <c r="H2" s="6" t="s">
         <v>147</v>
       </c>
-      <c r="I2" s="5" t="s">
+      <c r="I2" s="6" t="s">
         <v>148</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="6" t="s">
         <v>149</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="6" t="s">
         <v>150</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="6" t="s">
         <v>151</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="E3" s="6" t="s">
         <v>152</v>
       </c>
-      <c r="F3" s="5" t="s">
+      <c r="F3" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="G3" s="5" t="s">
+      <c r="G3" s="6" t="s">
         <v>153</v>
       </c>
-      <c r="H3" s="5" t="s">
+      <c r="H3" s="6" t="s">
         <v>154</v>
       </c>
-      <c r="I3" s="5" t="s">
+      <c r="I3" s="6" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="6" t="s">
         <v>156</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="6" t="s">
         <v>157</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="6" t="s">
         <v>158</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="E4" s="6" t="s">
         <v>159</v>
       </c>
-      <c r="F4" s="5" t="s">
+      <c r="F4" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="G4" s="5" t="s">
+      <c r="G4" s="6" t="s">
         <v>160</v>
       </c>
-      <c r="H4" s="5" t="s">
+      <c r="H4" s="6" t="s">
         <v>161</v>
       </c>
-      <c r="I4" s="5" t="s">
+      <c r="I4" s="6" t="s">
         <v>161</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="6" t="s">
         <v>162</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="6" t="s">
         <v>126</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D5" s="6" t="s">
         <v>163</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="E5" s="6" t="s">
         <v>164</v>
       </c>
-      <c r="F5" s="5"/>
-      <c r="G5" s="5" t="s">
+      <c r="F5" s="6"/>
+      <c r="G5" s="6" t="s">
         <v>165</v>
       </c>
-      <c r="H5" s="5" t="s">
+      <c r="H5" s="6" t="s">
         <v>166</v>
       </c>
-      <c r="I5" s="5" t="s">
+      <c r="I5" s="6" t="s">
         <v>167</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="6" t="s">
         <v>168</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="6" t="s">
         <v>169</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="D6" s="6" t="s">
         <v>170</v>
       </c>
-      <c r="E6" s="5" t="s">
+      <c r="E6" s="6" t="s">
         <v>171</v>
       </c>
-      <c r="F6" s="5"/>
-      <c r="G6" s="5" t="s">
+      <c r="F6" s="6"/>
+      <c r="G6" s="6" t="s">
         <v>172</v>
       </c>
-      <c r="H6" s="5" t="s">
+      <c r="H6" s="6" t="s">
         <v>173</v>
       </c>
-      <c r="I6" s="5" t="s">
+      <c r="I6" s="6" t="s">
         <v>174</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="s">
+      <c r="A7" s="6" t="s">
         <v>175</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="6" t="s">
         <v>176</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="C7" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="D7" s="6" t="s">
         <v>177</v>
       </c>
-      <c r="E7" s="5" t="s">
+      <c r="E7" s="6" t="s">
         <v>178</v>
       </c>
-      <c r="F7" s="5" t="s">
+      <c r="F7" s="6" t="s">
         <v>179</v>
       </c>
-      <c r="G7" s="5" t="s">
+      <c r="G7" s="6" t="s">
         <v>180</v>
       </c>
-      <c r="H7" s="5" t="s">
+      <c r="H7" s="6" t="s">
         <v>181</v>
       </c>
-      <c r="I7" s="5" t="s">
+      <c r="I7" s="6" t="s">
         <v>182</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="s">
+      <c r="A8" s="6" t="s">
         <v>183</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="C8" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="D8" s="6" t="s">
         <v>184</v>
       </c>
-      <c r="E8" s="5" t="s">
+      <c r="E8" s="6" t="s">
         <v>185</v>
       </c>
-      <c r="F8" s="5"/>
-      <c r="G8" s="5" t="s">
+      <c r="F8" s="6"/>
+      <c r="G8" s="6" t="s">
         <v>186</v>
       </c>
-      <c r="H8" s="5" t="s">
+      <c r="H8" s="6" t="s">
         <v>187</v>
       </c>
-      <c r="I8" s="5" t="s">
+      <c r="I8" s="6" t="s">
         <v>188</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="s">
+      <c r="A9" s="6" t="s">
         <v>189</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="C9" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="D9" s="5" t="s">
+      <c r="D9" s="6" t="s">
         <v>190</v>
       </c>
-      <c r="E9" s="5" t="s">
+      <c r="E9" s="6" t="s">
         <v>185</v>
       </c>
-      <c r="F9" s="5"/>
-      <c r="G9" s="5"/>
-      <c r="H9" s="5"/>
-      <c r="I9" s="5" t="s">
+      <c r="F9" s="6"/>
+      <c r="G9" s="6"/>
+      <c r="H9" s="6"/>
+      <c r="I9" s="6" t="s">
         <v>191</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="s">
+      <c r="A10" s="6" t="s">
         <v>192</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="B10" s="6" t="s">
         <v>193</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="C10" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="D10" s="5" t="s">
+      <c r="D10" s="6" t="s">
         <v>194</v>
       </c>
-      <c r="E10" s="5" t="s">
+      <c r="E10" s="6" t="s">
         <v>195</v>
       </c>
-      <c r="F10" s="5" t="s">
+      <c r="F10" s="6" t="s">
         <v>196</v>
       </c>
-      <c r="G10" s="5" t="s">
+      <c r="G10" s="6" t="s">
         <v>197</v>
       </c>
-      <c r="H10" s="5" t="s">
+      <c r="H10" s="6" t="s">
         <v>198</v>
       </c>
-      <c r="I10" s="5" t="s">
+      <c r="I10" s="6" t="s">
         <v>199</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="s">
+      <c r="A11" s="6" t="s">
         <v>200</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="B11" s="6" t="s">
         <v>126</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="C11" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="D11" s="5" t="s">
+      <c r="D11" s="6" t="s">
         <v>201</v>
       </c>
-      <c r="E11" s="5" t="s">
+      <c r="E11" s="6" t="s">
         <v>202</v>
       </c>
-      <c r="F11" s="5" t="s">
+      <c r="F11" s="6" t="s">
         <v>113</v>
       </c>
-      <c r="G11" s="5" t="s">
+      <c r="G11" s="6" t="s">
         <v>203</v>
       </c>
-      <c r="H11" s="5" t="s">
+      <c r="H11" s="6" t="s">
         <v>204</v>
       </c>
-      <c r="I11" s="5" t="s">
+      <c r="I11" s="6" t="s">
         <v>205</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="s">
+      <c r="A12" s="6" t="s">
         <v>137</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="B12" s="6" t="s">
         <v>138</v>
       </c>
-      <c r="C12" s="5" t="s">
+      <c r="C12" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="D12" s="5" t="s">
+      <c r="D12" s="6" t="s">
         <v>206</v>
       </c>
-      <c r="E12" s="5" t="s">
+      <c r="E12" s="6" t="s">
         <v>140</v>
       </c>
-      <c r="F12" s="5" t="s">
+      <c r="F12" s="6" t="s">
         <v>141</v>
       </c>
-      <c r="G12" s="5"/>
-      <c r="H12" s="5" t="s">
+      <c r="G12" s="6"/>
+      <c r="H12" s="6" t="s">
         <v>207</v>
       </c>
-      <c r="I12" s="5" t="s">
+      <c r="I12" s="6" t="s">
         <v>208</v>
       </c>
     </row>
@@ -11455,403 +11482,403 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="G1" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="H1" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="I1" s="5" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="C2" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="D2" s="6" t="s">
         <v>209</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="E2" s="6" t="s">
         <v>145</v>
       </c>
-      <c r="F2" s="5"/>
-      <c r="G2" s="5" t="s">
+      <c r="F2" s="6"/>
+      <c r="G2" s="6" t="s">
         <v>210</v>
       </c>
-      <c r="H2" s="5" t="s">
+      <c r="H2" s="6" t="s">
         <v>211</v>
       </c>
-      <c r="I2" s="5" t="s">
+      <c r="I2" s="6" t="s">
         <v>212</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="E3" s="6" t="s">
         <v>213</v>
       </c>
-      <c r="F3" s="5" t="s">
+      <c r="F3" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="G3" s="5" t="s">
+      <c r="G3" s="6" t="s">
         <v>214</v>
       </c>
-      <c r="H3" s="5" t="s">
+      <c r="H3" s="6" t="s">
         <v>215</v>
       </c>
-      <c r="I3" s="5" t="s">
+      <c r="I3" s="6" t="s">
         <v>216</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="6" t="s">
         <v>217</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="6" t="s">
         <v>218</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="6" t="s">
         <v>219</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="E4" s="6" t="s">
         <v>220</v>
       </c>
-      <c r="F4" s="5" t="s">
+      <c r="F4" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="G4" s="5" t="s">
+      <c r="G4" s="6" t="s">
         <v>221</v>
       </c>
-      <c r="H4" s="5" t="s">
+      <c r="H4" s="6" t="s">
         <v>222</v>
       </c>
-      <c r="I4" s="5" t="s">
+      <c r="I4" s="6" t="s">
         <v>223</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="6" t="s">
         <v>224</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>225</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>185</v>
+      </c>
+      <c r="F5" s="6"/>
+      <c r="G5" s="6" t="s">
+        <v>226</v>
+      </c>
+      <c r="H5" s="6" t="s">
+        <v>227</v>
+      </c>
+      <c r="I5" s="6" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="s">
+        <v>229</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="C6" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="D5" s="5" t="s">
-        <v>225</v>
-      </c>
-      <c r="E5" s="5" t="s">
+      <c r="D6" s="6" t="s">
+        <v>230</v>
+      </c>
+      <c r="E6" s="6" t="s">
         <v>185</v>
       </c>
-      <c r="F5" s="5"/>
-      <c r="G5" s="5" t="s">
-        <v>226</v>
-      </c>
-      <c r="H5" s="5" t="s">
-        <v>227</v>
-      </c>
-      <c r="I5" s="5" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="5" t="s">
-        <v>229</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="C6" s="5" t="s">
+      <c r="F6" s="6"/>
+      <c r="G6" s="6" t="s">
+        <v>231</v>
+      </c>
+      <c r="H6" s="6" t="s">
+        <v>232</v>
+      </c>
+      <c r="I6" s="6" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="s">
+        <v>175</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>176</v>
+      </c>
+      <c r="C7" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="D6" s="5" t="s">
-        <v>230</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>185</v>
-      </c>
-      <c r="F6" s="5"/>
-      <c r="G6" s="5" t="s">
-        <v>231</v>
-      </c>
-      <c r="H6" s="5" t="s">
-        <v>232</v>
-      </c>
-      <c r="I6" s="5" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="5" t="s">
-        <v>175</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>176</v>
-      </c>
-      <c r="C7" s="5" t="s">
+      <c r="D7" s="6" t="s">
+        <v>234</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>178</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="G7" s="6" t="s">
+        <v>235</v>
+      </c>
+      <c r="H7" s="6" t="s">
+        <v>236</v>
+      </c>
+      <c r="I7" s="6" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="s">
+        <v>192</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>193</v>
+      </c>
+      <c r="C8" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="D7" s="5" t="s">
-        <v>234</v>
-      </c>
-      <c r="E7" s="5" t="s">
-        <v>178</v>
-      </c>
-      <c r="F7" s="5" t="s">
-        <v>179</v>
-      </c>
-      <c r="G7" s="5" t="s">
-        <v>235</v>
-      </c>
-      <c r="H7" s="5" t="s">
-        <v>236</v>
-      </c>
-      <c r="I7" s="5" t="s">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="5" t="s">
-        <v>192</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>193</v>
-      </c>
-      <c r="C8" s="5" t="s">
+      <c r="D8" s="6" t="s">
+        <v>238</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>195</v>
+      </c>
+      <c r="F8" s="6" t="s">
+        <v>196</v>
+      </c>
+      <c r="G8" s="6" t="s">
+        <v>239</v>
+      </c>
+      <c r="H8" s="6" t="s">
+        <v>240</v>
+      </c>
+      <c r="I8" s="6" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="s">
+        <v>242</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="C9" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="D8" s="5" t="s">
-        <v>238</v>
-      </c>
-      <c r="E8" s="5" t="s">
-        <v>195</v>
-      </c>
-      <c r="F8" s="5" t="s">
-        <v>196</v>
-      </c>
-      <c r="G8" s="5" t="s">
-        <v>239</v>
-      </c>
-      <c r="H8" s="5" t="s">
-        <v>240</v>
-      </c>
-      <c r="I8" s="5" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="5" t="s">
-        <v>242</v>
-      </c>
-      <c r="B9" s="5" t="s">
+      <c r="D9" s="6" t="s">
+        <v>243</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="F9" s="6"/>
+      <c r="G9" s="6" t="s">
+        <v>244</v>
+      </c>
+      <c r="H9" s="6" t="s">
+        <v>245</v>
+      </c>
+      <c r="I9" s="6" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="s">
+        <v>247</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>248</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>249</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>250</v>
+      </c>
+      <c r="F10" s="6"/>
+      <c r="G10" s="6" t="s">
+        <v>251</v>
+      </c>
+      <c r="H10" s="6" t="s">
+        <v>252</v>
+      </c>
+      <c r="I10" s="6" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="s">
+        <v>254</v>
+      </c>
+      <c r="B11" s="6" t="s">
         <v>126</v>
       </c>
-      <c r="C9" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>243</v>
-      </c>
-      <c r="E9" s="5" t="s">
-        <v>105</v>
-      </c>
-      <c r="F9" s="5"/>
-      <c r="G9" s="5" t="s">
-        <v>244</v>
-      </c>
-      <c r="H9" s="5" t="s">
-        <v>245</v>
-      </c>
-      <c r="I9" s="5" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="5" t="s">
-        <v>247</v>
-      </c>
-      <c r="B10" s="5" t="s">
-        <v>248</v>
-      </c>
-      <c r="C10" s="5" t="s">
+      <c r="C11" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="D10" s="5" t="s">
-        <v>249</v>
-      </c>
-      <c r="E10" s="5" t="s">
-        <v>250</v>
-      </c>
-      <c r="F10" s="5"/>
-      <c r="G10" s="5" t="s">
-        <v>251</v>
-      </c>
-      <c r="H10" s="5" t="s">
-        <v>252</v>
-      </c>
-      <c r="I10" s="5" t="s">
-        <v>253</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="5" t="s">
-        <v>254</v>
-      </c>
-      <c r="B11" s="5" t="s">
+      <c r="D11" s="6" t="s">
+        <v>255</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>256</v>
+      </c>
+      <c r="F11" s="6"/>
+      <c r="G11" s="6" t="s">
+        <v>257</v>
+      </c>
+      <c r="H11" s="6" t="s">
+        <v>258</v>
+      </c>
+      <c r="I11" s="6" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="s">
+        <v>260</v>
+      </c>
+      <c r="B12" s="6" t="s">
         <v>126</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="C12" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="D11" s="5" t="s">
-        <v>255</v>
-      </c>
-      <c r="E11" s="5" t="s">
-        <v>256</v>
-      </c>
-      <c r="F11" s="5"/>
-      <c r="G11" s="5" t="s">
-        <v>257</v>
-      </c>
-      <c r="H11" s="5" t="s">
-        <v>258</v>
-      </c>
-      <c r="I11" s="5" t="s">
-        <v>259</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="5" t="s">
-        <v>260</v>
-      </c>
-      <c r="B12" s="5" t="s">
+      <c r="D12" s="6" t="s">
+        <v>261</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>262</v>
+      </c>
+      <c r="F12" s="6"/>
+      <c r="G12" s="6"/>
+      <c r="H12" s="6"/>
+      <c r="I12" s="6" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="s">
+        <v>200</v>
+      </c>
+      <c r="B13" s="6" t="s">
         <v>126</v>
       </c>
-      <c r="C12" s="5" t="s">
+      <c r="C13" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="D12" s="5" t="s">
-        <v>261</v>
-      </c>
-      <c r="E12" s="5" t="s">
-        <v>262</v>
-      </c>
-      <c r="F12" s="5"/>
-      <c r="G12" s="5"/>
-      <c r="H12" s="5"/>
-      <c r="I12" s="5" t="s">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="5" t="s">
-        <v>200</v>
-      </c>
-      <c r="B13" s="5" t="s">
+      <c r="D13" s="6" t="s">
+        <v>264</v>
+      </c>
+      <c r="E13" s="6" t="s">
+        <v>265</v>
+      </c>
+      <c r="F13" s="6"/>
+      <c r="G13" s="6"/>
+      <c r="H13" s="6"/>
+      <c r="I13" s="6"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="s">
+        <v>266</v>
+      </c>
+      <c r="B14" s="6" t="s">
         <v>126</v>
       </c>
-      <c r="C13" s="5" t="s">
+      <c r="C14" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="D13" s="5" t="s">
-        <v>264</v>
-      </c>
-      <c r="E13" s="5" t="s">
-        <v>265</v>
-      </c>
-      <c r="F13" s="5"/>
-      <c r="G13" s="5"/>
-      <c r="H13" s="5"/>
-      <c r="I13" s="5"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="5" t="s">
-        <v>266</v>
-      </c>
-      <c r="B14" s="5" t="s">
-        <v>126</v>
-      </c>
-      <c r="C14" s="5" t="s">
+      <c r="D14" s="6" t="s">
+        <v>267</v>
+      </c>
+      <c r="E14" s="6" t="s">
+        <v>268</v>
+      </c>
+      <c r="F14" s="6"/>
+      <c r="G14" s="6"/>
+      <c r="H14" s="6"/>
+      <c r="I14" s="6"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="C15" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="D14" s="5" t="s">
-        <v>267</v>
-      </c>
-      <c r="E14" s="5" t="s">
-        <v>268</v>
-      </c>
-      <c r="F14" s="5"/>
-      <c r="G14" s="5"/>
-      <c r="H14" s="5"/>
-      <c r="I14" s="5"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="5" t="s">
-        <v>137</v>
-      </c>
-      <c r="B15" s="5" t="s">
-        <v>138</v>
-      </c>
-      <c r="C15" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="D15" s="5" t="s">
+      <c r="D15" s="6" t="s">
         <v>269</v>
       </c>
-      <c r="E15" s="5" t="s">
+      <c r="E15" s="6" t="s">
         <v>140</v>
       </c>
-      <c r="F15" s="5" t="s">
+      <c r="F15" s="6" t="s">
         <v>141</v>
       </c>
-      <c r="G15" s="5" t="s">
+      <c r="G15" s="6" t="s">
         <v>270</v>
       </c>
-      <c r="H15" s="5" t="s">
+      <c r="H15" s="6" t="s">
         <v>271</v>
       </c>
-      <c r="I15" s="5" t="s">
+      <c r="I15" s="6" t="s">
         <v>272</v>
       </c>
     </row>
@@ -12861,195 +12888,195 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="G1" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="H1" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="I1" s="5" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="6" t="s">
         <v>273</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="C2" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="D2" s="6" t="s">
         <v>274</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="E2" s="6" t="s">
         <v>145</v>
       </c>
-      <c r="F2" s="5"/>
-      <c r="G2" s="5" t="s">
+      <c r="F2" s="6"/>
+      <c r="G2" s="6" t="s">
         <v>275</v>
       </c>
-      <c r="H2" s="5" t="s">
+      <c r="H2" s="6" t="s">
         <v>276</v>
       </c>
-      <c r="I2" s="5" t="s">
+      <c r="I2" s="6" t="s">
         <v>277</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="6" t="s">
         <v>278</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="6" t="s">
         <v>279</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="E3" s="6" t="s">
         <v>280</v>
       </c>
-      <c r="F3" s="5"/>
-      <c r="G3" s="5" t="s">
+      <c r="F3" s="6"/>
+      <c r="G3" s="6" t="s">
         <v>281</v>
       </c>
-      <c r="H3" s="5" t="s">
+      <c r="H3" s="6" t="s">
         <v>282</v>
       </c>
-      <c r="I3" s="5" t="s">
+      <c r="I3" s="6" t="s">
         <v>283</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="6" t="s">
         <v>284</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="6" t="s">
         <v>285</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="6" t="s">
         <v>286</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="E4" s="6" t="s">
         <v>287</v>
       </c>
-      <c r="F4" s="5" t="s">
+      <c r="F4" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="G4" s="5" t="s">
+      <c r="G4" s="6" t="s">
         <v>288</v>
       </c>
-      <c r="H4" s="5" t="s">
+      <c r="H4" s="6" t="s">
         <v>289</v>
       </c>
-      <c r="I4" s="5" t="s">
+      <c r="I4" s="6" t="s">
         <v>288</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="6" t="s">
         <v>290</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D5" s="6" t="s">
         <v>291</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="E5" s="6" t="s">
         <v>185</v>
       </c>
-      <c r="F5" s="5"/>
-      <c r="G5" s="5" t="s">
+      <c r="F5" s="6"/>
+      <c r="G5" s="6" t="s">
         <v>292</v>
       </c>
-      <c r="H5" s="5" t="s">
+      <c r="H5" s="6" t="s">
         <v>293</v>
       </c>
-      <c r="I5" s="5" t="s">
+      <c r="I5" s="6" t="s">
         <v>294</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="6" t="s">
         <v>229</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="D6" s="6" t="s">
         <v>295</v>
       </c>
-      <c r="E6" s="5" t="s">
+      <c r="E6" s="6" t="s">
         <v>185</v>
       </c>
-      <c r="F6" s="5"/>
-      <c r="G6" s="5" t="s">
+      <c r="F6" s="6"/>
+      <c r="G6" s="6" t="s">
         <v>296</v>
       </c>
-      <c r="H6" s="5" t="s">
+      <c r="H6" s="6" t="s">
         <v>297</v>
       </c>
-      <c r="I6" s="5" t="s">
+      <c r="I6" s="6" t="s">
         <v>298</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="s">
+      <c r="A7" s="6" t="s">
         <v>137</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="6" t="s">
         <v>138</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="C7" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="D7" s="6" t="s">
         <v>299</v>
       </c>
-      <c r="E7" s="5" t="s">
+      <c r="E7" s="6" t="s">
         <v>140</v>
       </c>
-      <c r="F7" s="5" t="s">
+      <c r="F7" s="6" t="s">
         <v>141</v>
       </c>
-      <c r="G7" s="5"/>
-      <c r="H7" s="5" t="s">
+      <c r="G7" s="6"/>
+      <c r="H7" s="6" t="s">
         <v>300</v>
       </c>
-      <c r="I7" s="5" t="s">
+      <c r="I7" s="6" t="s">
         <v>301</v>
       </c>
     </row>
@@ -14060,245 +14087,245 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="G1" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="H1" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="I1" s="5" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="C2" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="D2" s="6" t="s">
         <v>302</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="E2" s="6" t="s">
         <v>145</v>
       </c>
-      <c r="F2" s="5"/>
-      <c r="G2" s="5" t="s">
+      <c r="F2" s="6"/>
+      <c r="G2" s="6" t="s">
         <v>303</v>
       </c>
-      <c r="H2" s="5" t="s">
+      <c r="H2" s="6" t="s">
         <v>304</v>
       </c>
-      <c r="I2" s="5" t="s">
+      <c r="I2" s="6" t="s">
         <v>305</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="6" t="s">
         <v>224</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="6" t="s">
         <v>306</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="E3" s="6" t="s">
         <v>185</v>
       </c>
-      <c r="F3" s="5"/>
-      <c r="G3" s="5" t="s">
+      <c r="F3" s="6"/>
+      <c r="G3" s="6" t="s">
         <v>307</v>
       </c>
-      <c r="H3" s="5" t="s">
+      <c r="H3" s="6" t="s">
         <v>308</v>
       </c>
-      <c r="I3" s="5" t="s">
+      <c r="I3" s="6" t="s">
         <v>309</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="6" t="s">
         <v>310</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="6" t="s">
         <v>311</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="E4" s="6" t="s">
         <v>185</v>
       </c>
-      <c r="F4" s="5"/>
-      <c r="G4" s="5" t="s">
+      <c r="F4" s="6"/>
+      <c r="G4" s="6" t="s">
         <v>312</v>
       </c>
-      <c r="H4" s="5" t="s">
+      <c r="H4" s="6" t="s">
         <v>313</v>
       </c>
-      <c r="I4" s="5" t="s">
+      <c r="I4" s="6" t="s">
         <v>309</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D5" s="6" t="s">
         <v>314</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="E5" s="6" t="s">
         <v>213</v>
       </c>
-      <c r="F5" s="5" t="s">
+      <c r="F5" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="G5" s="5"/>
-      <c r="H5" s="5"/>
-      <c r="I5" s="5"/>
+      <c r="G5" s="6"/>
+      <c r="H5" s="6"/>
+      <c r="I5" s="6"/>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="6" t="s">
         <v>278</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="D6" s="6" t="s">
         <v>315</v>
       </c>
-      <c r="E6" s="5" t="s">
+      <c r="E6" s="6" t="s">
         <v>316</v>
       </c>
-      <c r="F6" s="5"/>
-      <c r="G6" s="5" t="s">
+      <c r="F6" s="6"/>
+      <c r="G6" s="6" t="s">
         <v>317</v>
       </c>
-      <c r="H6" s="5" t="s">
+      <c r="H6" s="6" t="s">
         <v>318</v>
       </c>
-      <c r="I6" s="5" t="s">
+      <c r="I6" s="6" t="s">
         <v>319</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="s">
+      <c r="A7" s="6" t="s">
         <v>229</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="C7" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="D7" s="6" t="s">
         <v>320</v>
       </c>
-      <c r="E7" s="5" t="s">
+      <c r="E7" s="6" t="s">
         <v>185</v>
       </c>
-      <c r="F7" s="5"/>
-      <c r="G7" s="5" t="s">
+      <c r="F7" s="6"/>
+      <c r="G7" s="6" t="s">
         <v>321</v>
       </c>
-      <c r="H7" s="5" t="s">
+      <c r="H7" s="6" t="s">
         <v>322</v>
       </c>
-      <c r="I7" s="5" t="s">
+      <c r="I7" s="6" t="s">
         <v>323</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="s">
+      <c r="A8" s="6" t="s">
         <v>324</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="6" t="s">
         <v>325</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="C8" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="D8" s="6" t="s">
         <v>326</v>
       </c>
-      <c r="E8" s="5" t="s">
+      <c r="E8" s="6" t="s">
         <v>327</v>
       </c>
-      <c r="F8" s="5"/>
-      <c r="G8" s="5" t="s">
+      <c r="F8" s="6"/>
+      <c r="G8" s="6" t="s">
         <v>328</v>
       </c>
-      <c r="H8" s="5" t="s">
+      <c r="H8" s="6" t="s">
         <v>329</v>
       </c>
-      <c r="I8" s="5" t="s">
+      <c r="I8" s="6" t="s">
         <v>330</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="s">
+      <c r="A9" s="6" t="s">
         <v>175</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="6" t="s">
         <v>176</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="C9" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="D9" s="5" t="s">
+      <c r="D9" s="6" t="s">
         <v>331</v>
       </c>
-      <c r="E9" s="5" t="s">
+      <c r="E9" s="6" t="s">
         <v>178</v>
       </c>
-      <c r="F9" s="5" t="s">
+      <c r="F9" s="6" t="s">
         <v>179</v>
       </c>
-      <c r="G9" s="5" t="s">
+      <c r="G9" s="6" t="s">
         <v>332</v>
       </c>
-      <c r="H9" s="5" t="s">
+      <c r="H9" s="6" t="s">
         <v>333</v>
       </c>
-      <c r="I9" s="5" t="s">
+      <c r="I9" s="6" t="s">
         <v>334</v>
       </c>
     </row>
@@ -15310,162 +15337,162 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="G1" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="H1" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="I1" s="5" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="6" t="s">
         <v>335</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="C2" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="D2" s="6" t="s">
         <v>336</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="E2" s="6" t="s">
         <v>337</v>
       </c>
-      <c r="F2" s="5" t="s">
+      <c r="F2" s="6" t="s">
         <v>196</v>
       </c>
-      <c r="G2" s="5" t="s">
+      <c r="G2" s="6" t="s">
         <v>303</v>
       </c>
-      <c r="H2" s="5" t="s">
+      <c r="H2" s="6" t="s">
         <v>338</v>
       </c>
-      <c r="I2" s="5" t="s">
+      <c r="I2" s="6" t="s">
         <v>339</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="6" t="s">
         <v>340</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="6" t="s">
         <v>341</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="E3" s="6" t="s">
         <v>185</v>
       </c>
-      <c r="F3" s="5"/>
-      <c r="G3" s="5" t="s">
+      <c r="F3" s="6"/>
+      <c r="G3" s="6" t="s">
         <v>307</v>
       </c>
-      <c r="H3" s="5" t="s">
+      <c r="H3" s="6" t="s">
         <v>342</v>
       </c>
-      <c r="I3" s="5" t="s">
+      <c r="I3" s="6" t="s">
         <v>343</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="6" t="s">
         <v>344</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="6" t="s">
         <v>345</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="6" t="s">
         <v>346</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="E4" s="6" t="s">
         <v>347</v>
       </c>
-      <c r="F4" s="5" t="s">
+      <c r="F4" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="G4" s="5" t="s">
+      <c r="G4" s="6" t="s">
         <v>348</v>
       </c>
-      <c r="H4" s="5" t="s">
+      <c r="H4" s="6" t="s">
         <v>349</v>
       </c>
-      <c r="I4" s="5" t="s">
+      <c r="I4" s="6" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="6" t="s">
         <v>350</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D5" s="6" t="s">
         <v>351</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="E5" s="6" t="s">
         <v>352</v>
       </c>
-      <c r="F5" s="5"/>
-      <c r="G5" s="5"/>
-      <c r="H5" s="5"/>
-      <c r="I5" s="5"/>
+      <c r="F5" s="6"/>
+      <c r="G5" s="6"/>
+      <c r="H5" s="6"/>
+      <c r="I5" s="6"/>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="D6" s="6" t="s">
         <v>353</v>
       </c>
-      <c r="E6" s="5" t="s">
+      <c r="E6" s="6" t="s">
         <v>213</v>
       </c>
-      <c r="F6" s="5" t="s">
+      <c r="F6" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="G6" s="5"/>
-      <c r="H6" s="5"/>
-      <c r="I6" s="5"/>
+      <c r="G6" s="6"/>
+      <c r="H6" s="6"/>
+      <c r="I6" s="6"/>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
     <row r="22" ht="15.75" customHeight="1"/>
@@ -16474,187 +16501,187 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="G1" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="H1" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="I1" s="5" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="6" t="s">
         <v>354</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="6" t="s">
         <v>355</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="C2" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="D2" s="6" t="s">
         <v>356</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="E2" s="6" t="s">
         <v>357</v>
       </c>
-      <c r="F2" s="5"/>
-      <c r="G2" s="5" t="s">
+      <c r="F2" s="6"/>
+      <c r="G2" s="6" t="s">
         <v>358</v>
       </c>
-      <c r="H2" s="5" t="s">
+      <c r="H2" s="6" t="s">
         <v>358</v>
       </c>
-      <c r="I2" s="5" t="s">
+      <c r="I2" s="6" t="s">
         <v>359</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="6" t="s">
         <v>360</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="6" t="s">
         <v>361</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="E3" s="6" t="s">
         <v>362</v>
       </c>
-      <c r="F3" s="5"/>
-      <c r="G3" s="5" t="s">
+      <c r="F3" s="6"/>
+      <c r="G3" s="6" t="s">
         <v>363</v>
       </c>
-      <c r="H3" s="5" t="s">
+      <c r="H3" s="6" t="s">
         <v>364</v>
       </c>
-      <c r="I3" s="5" t="s">
+      <c r="I3" s="6" t="s">
         <v>365</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="6" t="s">
         <v>366</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="6" t="s">
         <v>355</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="6" t="s">
         <v>367</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="E4" s="6" t="s">
         <v>368</v>
       </c>
-      <c r="F4" s="5"/>
-      <c r="G4" s="5"/>
-      <c r="H4" s="5" t="s">
+      <c r="F4" s="6"/>
+      <c r="G4" s="6"/>
+      <c r="H4" s="6" t="s">
         <v>369</v>
       </c>
-      <c r="I4" s="5" t="s">
+      <c r="I4" s="6" t="s">
         <v>370</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="6" t="s">
         <v>371</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D5" s="6" t="s">
         <v>372</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="E5" s="6" t="s">
         <v>373</v>
       </c>
-      <c r="F5" s="5"/>
-      <c r="G5" s="5"/>
-      <c r="H5" s="5" t="s">
+      <c r="F5" s="6"/>
+      <c r="G5" s="6"/>
+      <c r="H5" s="6" t="s">
         <v>374</v>
       </c>
-      <c r="I5" s="5" t="s">
+      <c r="I5" s="6" t="s">
         <v>375</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="6" t="s">
         <v>376</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="D6" s="6" t="s">
         <v>377</v>
       </c>
-      <c r="E6" s="5" t="s">
+      <c r="E6" s="6" t="s">
         <v>185</v>
       </c>
-      <c r="F6" s="5"/>
-      <c r="G6" s="5"/>
-      <c r="H6" s="5" t="s">
+      <c r="F6" s="6"/>
+      <c r="G6" s="6"/>
+      <c r="H6" s="6" t="s">
         <v>378</v>
       </c>
-      <c r="I6" s="5" t="s">
+      <c r="I6" s="6" t="s">
         <v>379</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="s">
+      <c r="A7" s="6" t="s">
         <v>380</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="6" t="s">
         <v>381</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="C7" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="D7" s="6" t="s">
         <v>382</v>
       </c>
-      <c r="E7" s="5" t="s">
+      <c r="E7" s="6" t="s">
         <v>383</v>
       </c>
-      <c r="F7" s="5"/>
-      <c r="G7" s="5" t="s">
+      <c r="F7" s="6"/>
+      <c r="G7" s="6" t="s">
         <v>384</v>
       </c>
-      <c r="H7" s="5" t="s">
+      <c r="H7" s="6" t="s">
         <v>385</v>
       </c>
-      <c r="I7" s="5" t="s">
+      <c r="I7" s="6" t="s">
         <v>386</v>
       </c>
     </row>
@@ -17665,193 +17692,193 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="G1" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="H1" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="I1" s="5" t="s">
         <v>49</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="6" t="s">
         <v>387</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="6" t="s">
         <v>355</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="C2" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="D2" s="6" t="s">
         <v>388</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="E2" s="6" t="s">
         <v>389</v>
       </c>
-      <c r="F2" s="5"/>
-      <c r="G2" s="5" t="s">
+      <c r="F2" s="6"/>
+      <c r="G2" s="6" t="s">
         <v>390</v>
       </c>
-      <c r="H2" s="5" t="s">
+      <c r="H2" s="6" t="s">
         <v>391</v>
       </c>
-      <c r="I2" s="5" t="s">
+      <c r="I2" s="6" t="s">
         <v>392</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="6" t="s">
         <v>393</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="6" t="s">
         <v>394</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="E3" s="6" t="s">
         <v>395</v>
       </c>
-      <c r="F3" s="5"/>
-      <c r="G3" s="5" t="s">
+      <c r="F3" s="6"/>
+      <c r="G3" s="6" t="s">
         <v>390</v>
       </c>
-      <c r="H3" s="5" t="s">
+      <c r="H3" s="6" t="s">
         <v>396</v>
       </c>
-      <c r="I3" s="5" t="s">
+      <c r="I3" s="6" t="s">
         <v>396</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="6" t="s">
         <v>397</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="6" t="s">
         <v>398</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="E4" s="6" t="s">
         <v>185</v>
       </c>
-      <c r="F4" s="5"/>
-      <c r="G4" s="5" t="s">
+      <c r="F4" s="6"/>
+      <c r="G4" s="6" t="s">
         <v>390</v>
       </c>
-      <c r="H4" s="5" t="s">
+      <c r="H4" s="6" t="s">
         <v>399</v>
       </c>
-      <c r="I4" s="5" t="s">
+      <c r="I4" s="6" t="s">
         <v>400</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="6" t="s">
         <v>401</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="6" t="s">
         <v>355</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D5" s="6" t="s">
         <v>402</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="E5" s="6" t="s">
         <v>389</v>
       </c>
-      <c r="F5" s="5"/>
-      <c r="G5" s="5" t="s">
+      <c r="F5" s="6"/>
+      <c r="G5" s="6" t="s">
         <v>390</v>
       </c>
-      <c r="H5" s="5" t="s">
+      <c r="H5" s="6" t="s">
         <v>403</v>
       </c>
-      <c r="I5" s="5" t="s">
+      <c r="I5" s="6" t="s">
         <v>404</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="6" t="s">
         <v>405</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="D6" s="6" t="s">
         <v>406</v>
       </c>
-      <c r="E6" s="5" t="s">
+      <c r="E6" s="6" t="s">
         <v>185</v>
       </c>
-      <c r="F6" s="5"/>
-      <c r="G6" s="5" t="s">
+      <c r="F6" s="6"/>
+      <c r="G6" s="6" t="s">
         <v>390</v>
       </c>
-      <c r="H6" s="5" t="s">
+      <c r="H6" s="6" t="s">
         <v>407</v>
       </c>
-      <c r="I6" s="5" t="s">
+      <c r="I6" s="6" t="s">
         <v>408</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="s">
+      <c r="A7" s="6" t="s">
         <v>409</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="C7" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="D7" s="6" t="s">
         <v>410</v>
       </c>
-      <c r="E7" s="5" t="s">
+      <c r="E7" s="6" t="s">
         <v>185</v>
       </c>
-      <c r="F7" s="5"/>
-      <c r="G7" s="5" t="s">
+      <c r="F7" s="6"/>
+      <c r="G7" s="6" t="s">
         <v>390</v>
       </c>
-      <c r="H7" s="5" t="s">
+      <c r="H7" s="6" t="s">
         <v>411</v>
       </c>
-      <c r="I7" s="5" t="s">
+      <c r="I7" s="6" t="s">
         <v>412</v>
       </c>
     </row>

</xml_diff>